<commit_message>
feat: Luban cell.* 配置表落地（135 卡 / 30 敌人 / 28 技能 / 32 词缀）
13 张表 + 15 个枚举块，Luban codegen 通过，生成 14 个 Tb 类与 bytes。
内容量与 Cell_Stage_Spec.md §8.3 的分布目标一致：
- 稀有度 44 普通 / 44 稀有 / 25 史诗 / 15 异化 / 7 遗产
- 路线 22/22/22/19/19/18 + 13 跨路线联动
- 纯数值卡 12/135 = 8.9%，在 Spec §16 的 15% 上限内

DataRegistry.LoadFromLuban 改为真实实现（CellLubanLoader），
它是全工程唯一直接引用 GameConfig.cell.* 的地方——玩法代码只认本层
Spec 类型，所以配置源可整体替换。CellContentSeed 从表未就绪的临时内容
改为表损坏时的降级形态，注释已说明两者不同步是刻意的。

两个 Luban 约束踩坑记录（写进 gen_all.py 头部）：
不允许跨模块同名表，fp 已占 TbGlobal/TbEnemy，故 cell 侧叫 CellGlobal/CellEnemy。

生成器在 tools/cell_tables/，分 5 步且可一键重跑：
step5 做跨表引用自检（原型索引连续性、Spawn 指向的敌人是否存在、
异化/遗产卡是否漏填副作用、OnTick 卡 interval 是否为 0 会每帧触发、
Area 效果 duration 是否为 0 会退化成瞬时、每个时期可抽卡是否够 3 选 1 等）。
这类错误在生成期发现比运行时崩掉便宜得多。
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/__enums__.xlsx
+++ b/Configs/GameConfig/Datas/__enums__.xlsx
@@ -1092,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L212"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" style="4" min="2" max="2"/>
@@ -1780,84 +1780,3392 @@
       <c r="K31" s="0" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>fp.EEnemyId</t>
         </is>
       </c>
-      <c r="C32" t="b">
+      <c r="C32" s="0" t="b">
         <v>0</v>
       </c>
-      <c r="D32" t="b">
+      <c r="D32" s="0" t="b">
         <v>1</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="0" t="inlineStr">
         <is>
           <t>敌人类型</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H32" s="0" t="inlineStr">
         <is>
           <t>Threat</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="0" t="inlineStr">
         <is>
           <t>细胞威胁</t>
         </is>
       </c>
-      <c r="J32" t="n">
+      <c r="J32" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" s="0" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="0" t="inlineStr">
         <is>
           <t>Herbivore</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="0" t="inlineStr">
         <is>
           <t>草食虫</t>
         </is>
       </c>
-      <c r="J33" t="n">
+      <c r="J33" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" s="0" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="0" t="inlineStr">
         <is>
           <t>Predator</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="0" t="inlineStr">
         <is>
           <t>掠食虫</t>
         </is>
       </c>
-      <c r="J34" t="n">
+      <c r="J34" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" s="0" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="H35" t="inlineStr">
+      <c r="H35" s="0" t="inlineStr">
         <is>
           <t>Elite</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="0" t="inlineStr">
         <is>
           <t>精英</t>
         </is>
       </c>
-      <c r="J35" t="n">
+      <c r="J35" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" s="0" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>cell.ERoute</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>原型路线</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Devour</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>吞噬扩张</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Agile</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>机动猎食</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>2</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Electric</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>电化统治</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>3</v>
+      </c>
+      <c r="K39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Spore</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>孢子繁殖</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>4</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Nest</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>菌毯筑巢</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>5</v>
+      </c>
+      <c r="K41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Corrupt</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>异化污染</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>6</v>
+      </c>
+      <c r="K42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>跨路线联动</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>7</v>
+      </c>
+      <c r="K43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>cell.ERarity</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>卡牌稀有度</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>建立基础循环</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>稀有</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>形成路线联动</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>史诗</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>2</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>改变一条路线的运作方式</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Aberrant</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>异化</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>3</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>强机制变化 + 明确副作用</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>原核遗产</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>4</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>定义整局策略</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>cell.ETrigger</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>卡牌触发时机</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>获得即生效</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>OnDevour</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>吞噬时</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>OnKill</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>击杀时</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>OnHit</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>命中时</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>OnHurt</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>受伤时</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>4</v>
+      </c>
+      <c r="K53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>OnDash</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>冲刺时</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>5</v>
+      </c>
+      <c r="K54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>OnAbilityCast</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>施放技能时</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>6</v>
+      </c>
+      <c r="K55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>OnLevelUp</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>升级时</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>7</v>
+      </c>
+      <c r="K56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>OnLowHealth</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>低血时</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>8</v>
+      </c>
+      <c r="K57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>OnPhaseStart</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>时期开始时</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>9</v>
+      </c>
+      <c r="K58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>OnTick</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>周期性</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>10</v>
+      </c>
+      <c r="K59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>OnVolumeChanged</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>体积变化时</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>11</v>
+      </c>
+      <c r="K60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>OnEcoEvent</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>生态事件时</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>12</v>
+      </c>
+      <c r="K61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>cell.EEffectKind</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>效果类别</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Damage</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>2</v>
+      </c>
+      <c r="K64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Spawn</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>生成单位</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>3</v>
+      </c>
+      <c r="K65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>属性修正</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>4</v>
+      </c>
+      <c r="K66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>资源变化</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>5</v>
+      </c>
+      <c r="K67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Dash</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>位移</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>6</v>
+      </c>
+      <c r="K68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Projectile</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>投射物</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>7</v>
+      </c>
+      <c r="K69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>持续区域</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>8</v>
+      </c>
+      <c r="K70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>改规则</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>9</v>
+      </c>
+      <c r="K71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>cell.EEffectShape</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>效果形状</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>自身</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Circle</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>圆形</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>1</v>
+      </c>
+      <c r="K73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Cone</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>锥形</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>2</v>
+      </c>
+      <c r="K74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>直线</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>3</v>
+      </c>
+      <c r="K75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>单目标</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>4</v>
+      </c>
+      <c r="K76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>指定点</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>5</v>
+      </c>
+      <c r="K77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>cell.EAffix</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>词缀</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Proliferate</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>增殖</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>1</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>生成数量翻倍</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Conductive</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>导电</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>2</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>与电系联动</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Corrosive</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>腐蚀</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>3</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>持续削弱体积护壳速度</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Refund</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>回流</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>4</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>返还体力冷却营养</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Fission</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>裂变</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>5</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>结束时生成次级效果</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Mimic</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>拟态</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>6</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>复制上次触发的弱版</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Hunger</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>饥饿</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>7</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>低资源时更强</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Homeostasis</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>稳态</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>8</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>静止筑巢时更强</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Overload</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>过载</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>9</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>强化但自损</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Symbiosis</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>共生</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>10</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>附属体越多本体越强</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>贯穿</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>11</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>效果穿透目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Ricochet</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>弹射</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>12</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>命中后跳向下一目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Lingering</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>滞留</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>13</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>留下持续区域</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Gravity</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>引力</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>14</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>拉拽附近目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Fear</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>恐惧</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>15</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>逼退小型敌人</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>标记</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>16</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>施加易伤标记</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Parasite</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>寄生</t>
+        </is>
+      </c>
+      <c r="J95" t="n">
+        <v>17</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>附着并持续削弱</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Siphon</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>虹吸</t>
+        </is>
+      </c>
+      <c r="J96" t="n">
+        <v>18</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>转化敌方资源</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Harden</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>硬化</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>19</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>提高受击阈值</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Molt</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>蜕变</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>20</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>受击时转换形态</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Chain</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>连锁</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>21</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>触发次数递增</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Resonate</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>共振</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>22</v>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>多目标互相加成</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Delayed</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>淤积</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>23</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>效果延迟但加倍</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Catalyze</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>催化</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>24</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>缩短其他冷却</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>分食</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>25</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>大目标死亡裂成小块</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Hatch</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>孵化</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>26</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>延迟生成友方单位</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Crystallize</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>晶化</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>27</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>累积破碎层数</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Tidal</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>潮汐</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>28</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>周期性强弱交替</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>BoneEater</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>噬骨</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>29</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>对高体积目标增伤</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Detached</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>游离</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>30</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>效果可脱离本体存在</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Entropy</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>逆熵</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>31</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>消耗污染度换取回复</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Sacrifice</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>献祭</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>32</v>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>消耗自身资源大幅强化</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>cell.ERuleFlag</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>规则开关</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>CorpseEdible</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>尸体可食</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>1</v>
+      </c>
+      <c r="K112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>FailedDevourCorrodes</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>吞噬失败致腐蚀</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>2</v>
+      </c>
+      <c r="K113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>ComboNeverResets</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>连吃不清空</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>3</v>
+      </c>
+      <c r="K114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>DashPierces</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>冲刺穿体</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>4</v>
+      </c>
+      <c r="K115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>DashLeavesCurrent</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>冲刺留电流</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>5</v>
+      </c>
+      <c r="K116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>CorpseConducts</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>尸体导电</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>6</v>
+      </c>
+      <c r="K117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>MyceliumBoostsDevour</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>菌毯增益吞噬</t>
+        </is>
+      </c>
+      <c r="J118" t="n">
+        <v>7</v>
+      </c>
+      <c r="K118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>AutoEscapeOnLowHp</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>濒死脱战</t>
+        </is>
+      </c>
+      <c r="J119" t="n">
+        <v>8</v>
+      </c>
+      <c r="K119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>PollutionBecomesOverlord</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>污染满转霸主</t>
+        </is>
+      </c>
+      <c r="J120" t="n">
+        <v>9</v>
+      </c>
+      <c r="K120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>MinionsFocusMarked</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>附属体集火标记</t>
+        </is>
+      </c>
+      <c r="J121" t="n">
+        <v>10</v>
+      </c>
+      <c r="K121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>LargeTargetsSplit</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>大目标裂解</t>
+        </is>
+      </c>
+      <c r="J122" t="n">
+        <v>11</v>
+      </c>
+      <c r="K122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>ExecuteCausesFear</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>处决致恐惧</t>
+        </is>
+      </c>
+      <c r="J123" t="n">
+        <v>12</v>
+      </c>
+      <c r="K123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>cell.ETargetMode</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>技能瞄准方式</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Self</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>自身</t>
+        </is>
+      </c>
+      <c r="J124" t="n">
+        <v>0</v>
+      </c>
+      <c r="K124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>MoveDirection</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>移动方向</t>
+        </is>
+      </c>
+      <c r="J125" t="n">
+        <v>1</v>
+      </c>
+      <c r="K125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>鼠标方向</t>
+        </is>
+      </c>
+      <c r="J126" t="n">
+        <v>2</v>
+      </c>
+      <c r="K126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>NearestEnemy</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>最近敌人</t>
+        </is>
+      </c>
+      <c r="J127" t="n">
+        <v>3</v>
+      </c>
+      <c r="K127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>MarkedEnemy</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>已标记敌人</t>
+        </is>
+      </c>
+      <c r="J128" t="n">
+        <v>4</v>
+      </c>
+      <c r="K128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>cell.EStatId</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>属性 id</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J129" t="n">
+        <v>0</v>
+      </c>
+      <c r="K129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>MaxHealth</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>最大生命</t>
+        </is>
+      </c>
+      <c r="J130" t="n">
+        <v>1</v>
+      </c>
+      <c r="K130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>MoveSpeed</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>移速</t>
+        </is>
+      </c>
+      <c r="J131" t="n">
+        <v>2</v>
+      </c>
+      <c r="K131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>体积</t>
+        </is>
+      </c>
+      <c r="J132" t="n">
+        <v>3</v>
+      </c>
+      <c r="K132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>MeleeDamage</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>近战伤害</t>
+        </is>
+      </c>
+      <c r="J133" t="n">
+        <v>4</v>
+      </c>
+      <c r="K133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>DevourRatio</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>吞噬门槛</t>
+        </is>
+      </c>
+      <c r="J134" t="n">
+        <v>5</v>
+      </c>
+      <c r="K134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>DevourGain</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>吞噬收益</t>
+        </is>
+      </c>
+      <c r="J135" t="n">
+        <v>6</v>
+      </c>
+      <c r="K135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>StaminaMax</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>体力上限</t>
+        </is>
+      </c>
+      <c r="J136" t="n">
+        <v>7</v>
+      </c>
+      <c r="K136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>StaminaRegen</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>体力回复</t>
+        </is>
+      </c>
+      <c r="J137" t="n">
+        <v>8</v>
+      </c>
+      <c r="K137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>DashCost</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>冲刺消耗</t>
+        </is>
+      </c>
+      <c r="J138" t="n">
+        <v>9</v>
+      </c>
+      <c r="K138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>DashDistance</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>冲刺距离</t>
+        </is>
+      </c>
+      <c r="J139" t="n">
+        <v>10</v>
+      </c>
+      <c r="K139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>DashInvulnTime</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>冲刺无敌时长</t>
+        </is>
+      </c>
+      <c r="J140" t="n">
+        <v>11</v>
+      </c>
+      <c r="K140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>CooldownReduction</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>冷却缩减</t>
+        </is>
+      </c>
+      <c r="J141" t="n">
+        <v>12</v>
+      </c>
+      <c r="K141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>AreaScale</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>范围倍率</t>
+        </is>
+      </c>
+      <c r="J142" t="n">
+        <v>13</v>
+      </c>
+      <c r="K142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>AbilityPower</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>技能强度</t>
+        </is>
+      </c>
+      <c r="J143" t="n">
+        <v>14</v>
+      </c>
+      <c r="K143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>ElectricPower</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>电系强度</t>
+        </is>
+      </c>
+      <c r="J144" t="n">
+        <v>15</v>
+      </c>
+      <c r="K144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>ChainBonus</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>连锁加成</t>
+        </is>
+      </c>
+      <c r="J145" t="n">
+        <v>16</v>
+      </c>
+      <c r="K145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>MinionCap</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>附属体上限</t>
+        </is>
+      </c>
+      <c r="J146" t="n">
+        <v>17</v>
+      </c>
+      <c r="K146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>MinionPower</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>附属体强度</t>
+        </is>
+      </c>
+      <c r="J147" t="n">
+        <v>18</v>
+      </c>
+      <c r="K147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>HealthRegen</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>生命回复</t>
+        </is>
+      </c>
+      <c r="J148" t="n">
+        <v>19</v>
+      </c>
+      <c r="K148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>KillHeal</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>击杀回复</t>
+        </is>
+      </c>
+      <c r="J149" t="n">
+        <v>20</v>
+      </c>
+      <c r="K149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>DamageTaken</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>受伤倍率</t>
+        </is>
+      </c>
+      <c r="J150" t="n">
+        <v>21</v>
+      </c>
+      <c r="K150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>AggroScale</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>仇恨倍率</t>
+        </is>
+      </c>
+      <c r="J151" t="n">
+        <v>22</v>
+      </c>
+      <c r="K151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>PickupRadius</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>拾取半径</t>
+        </is>
+      </c>
+      <c r="J152" t="n">
+        <v>23</v>
+      </c>
+      <c r="K152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>EvoGain</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>进化能收益</t>
+        </is>
+      </c>
+      <c r="J153" t="n">
+        <v>24</v>
+      </c>
+      <c r="K153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>NutrientGain</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>营养质收益</t>
+        </is>
+      </c>
+      <c r="J154" t="n">
+        <v>25</v>
+      </c>
+      <c r="K154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>AbilitySlots</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>技能槽位</t>
+        </is>
+      </c>
+      <c r="J155" t="n">
+        <v>26</v>
+      </c>
+      <c r="K155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>PollutionCap</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>污染度上限</t>
+        </is>
+      </c>
+      <c r="J156" t="n">
+        <v>27</v>
+      </c>
+      <c r="K156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>MyceliumScale</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>菌毯范围</t>
+        </is>
+      </c>
+      <c r="J157" t="n">
+        <v>28</v>
+      </c>
+      <c r="K157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>ProjectileCount</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>投射物数量</t>
+        </is>
+      </c>
+      <c r="J158" t="n">
+        <v>29</v>
+      </c>
+      <c r="K158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>StatusDuration</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>状态时长</t>
+        </is>
+      </c>
+      <c r="J159" t="n">
+        <v>30</v>
+      </c>
+      <c r="K159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>cell.EModifierOp</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>修正器叠加层级</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>加值</t>
+        </is>
+      </c>
+      <c r="J160" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>PctAdd</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>加法百分比</t>
+        </is>
+      </c>
+      <c r="J161" t="n">
+        <v>1</v>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>同类相加</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>PctMul</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>乘法百分比</t>
+        </is>
+      </c>
+      <c r="J162" t="n">
+        <v>2</v>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>独立相乘</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>cell.EResourceKind</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>资源种类</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J163" t="n">
+        <v>0</v>
+      </c>
+      <c r="K163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>生命值</t>
+        </is>
+      </c>
+      <c r="J164" t="n">
+        <v>1</v>
+      </c>
+      <c r="K164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Nutrient</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>营养质</t>
+        </is>
+      </c>
+      <c r="J165" t="n">
+        <v>2</v>
+      </c>
+      <c r="K165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Mutagen</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>突变质</t>
+        </is>
+      </c>
+      <c r="J166" t="n">
+        <v>3</v>
+      </c>
+      <c r="K166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>EvoEnergy</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>进化能</t>
+        </is>
+      </c>
+      <c r="J167" t="n">
+        <v>4</v>
+      </c>
+      <c r="K167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Pollution</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>污染度</t>
+        </is>
+      </c>
+      <c r="J168" t="n">
+        <v>5</v>
+      </c>
+      <c r="K168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>体积</t>
+        </is>
+      </c>
+      <c r="J169" t="n">
+        <v>6</v>
+      </c>
+      <c r="K169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Stamina</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>体力</t>
+        </is>
+      </c>
+      <c r="J170" t="n">
+        <v>7</v>
+      </c>
+      <c r="K170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>cell.EDraftKind</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>选卡类型</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>常规升级</t>
+        </is>
+      </c>
+      <c r="J171" t="n">
+        <v>0</v>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>3 选 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>精英进化</t>
+        </is>
+      </c>
+      <c r="J172" t="n">
+        <v>1</v>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>4 选 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Corrupt</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>污染进化</t>
+        </is>
+      </c>
+      <c r="J173" t="n">
+        <v>2</v>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>3 选 1 带代价</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Repair</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>修复进化</t>
+        </is>
+      </c>
+      <c r="J174" t="n">
+        <v>3</v>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>2 选 1 保底</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>遗产进化</t>
+        </is>
+      </c>
+      <c r="J175" t="n">
+        <v>4</v>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>3 选 1 遗产卡</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>cell.EBehaviorKind</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>行为原型</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Stationary</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>固守</t>
+        </is>
+      </c>
+      <c r="J176" t="n">
+        <v>0</v>
+      </c>
+      <c r="K176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Drift</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>漂浮</t>
+        </is>
+      </c>
+      <c r="J177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Chase</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>追猎</t>
+        </is>
+      </c>
+      <c r="J178" t="n">
+        <v>2</v>
+      </c>
+      <c r="K178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Patrol</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>巡逻</t>
+        </is>
+      </c>
+      <c r="J179" t="n">
+        <v>3</v>
+      </c>
+      <c r="K179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Charge</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>冲撞</t>
+        </is>
+      </c>
+      <c r="J180" t="n">
+        <v>4</v>
+      </c>
+      <c r="K180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>远程</t>
+        </is>
+      </c>
+      <c r="J181" t="n">
+        <v>5</v>
+      </c>
+      <c r="K181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Swarm</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>群体</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v>6</v>
+      </c>
+      <c r="K182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Flee</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>逃逸</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>7</v>
+      </c>
+      <c r="K183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Orbit</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>环绕</t>
+        </is>
+      </c>
+      <c r="J184" t="n">
+        <v>8</v>
+      </c>
+      <c r="K184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Latch</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>附着</t>
+        </is>
+      </c>
+      <c r="J185" t="n">
+        <v>9</v>
+      </c>
+      <c r="K185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>cell.EStatus</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>状态位</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J186" t="n">
+        <v>0</v>
+      </c>
+      <c r="K186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Conductive</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>导电</t>
+        </is>
+      </c>
+      <c r="J187" t="n">
+        <v>1</v>
+      </c>
+      <c r="K187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Breached</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>破体</t>
+        </is>
+      </c>
+      <c r="J188" t="n">
+        <v>2</v>
+      </c>
+      <c r="K188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>标记</t>
+        </is>
+      </c>
+      <c r="J189" t="n">
+        <v>4</v>
+      </c>
+      <c r="K189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Slowed</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>减速</t>
+        </is>
+      </c>
+      <c r="J190" t="n">
+        <v>8</v>
+      </c>
+      <c r="K190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Stunned</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>麻痹</t>
+        </is>
+      </c>
+      <c r="J191" t="n">
+        <v>16</v>
+      </c>
+      <c r="K191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Corroded</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>腐蚀</t>
+        </is>
+      </c>
+      <c r="J192" t="n">
+        <v>32</v>
+      </c>
+      <c r="K192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Feared</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>恐惧</t>
+        </is>
+      </c>
+      <c r="J193" t="n">
+        <v>64</v>
+      </c>
+      <c r="K193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Parasited</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>寄生</t>
+        </is>
+      </c>
+      <c r="J194" t="n">
+        <v>128</v>
+      </c>
+      <c r="K194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Invulnerable</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>无敌</t>
+        </is>
+      </c>
+      <c r="J195" t="n">
+        <v>256</v>
+      </c>
+      <c r="K195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Hardened</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>硬化</t>
+        </is>
+      </c>
+      <c r="J196" t="n">
+        <v>512</v>
+      </c>
+      <c r="K196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Crystallized</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>晶化</t>
+        </is>
+      </c>
+      <c r="J197" t="n">
+        <v>1024</v>
+      </c>
+      <c r="K197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Infected</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>感染</t>
+        </is>
+      </c>
+      <c r="J198" t="n">
+        <v>2048</v>
+      </c>
+      <c r="K198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Vulnerable</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>易伤</t>
+        </is>
+      </c>
+      <c r="J199" t="n">
+        <v>4096</v>
+      </c>
+      <c r="K199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Burning</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>燃烧</t>
+        </is>
+      </c>
+      <c r="J200" t="n">
+        <v>8192</v>
+      </c>
+      <c r="K200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Polluted</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>污染</t>
+        </is>
+      </c>
+      <c r="J201" t="n">
+        <v>16384</v>
+      </c>
+      <c r="K201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Pulled</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>被拉拽</t>
+        </is>
+      </c>
+      <c r="J202" t="n">
+        <v>32768</v>
+      </c>
+      <c r="K202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Unedible</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>不可吞噬</t>
+        </is>
+      </c>
+      <c r="J203" t="n">
+        <v>65536</v>
+      </c>
+      <c r="K203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>精英</t>
+        </is>
+      </c>
+      <c r="J204" t="n">
+        <v>131072</v>
+      </c>
+      <c r="K204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>首领</t>
+        </is>
+      </c>
+      <c r="J205" t="n">
+        <v>262144</v>
+      </c>
+      <c r="K205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>OnMycelium</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>菌毯上</t>
+        </is>
+      </c>
+      <c r="J206" t="n">
+        <v>524288</v>
+      </c>
+      <c r="K206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>cell.EFaction</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>阵营</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="J207" t="n">
+        <v>0</v>
+      </c>
+      <c r="K207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>玩家</t>
+        </is>
+      </c>
+      <c r="J208" t="n">
+        <v>1</v>
+      </c>
+      <c r="K208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>PlayerMinion</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>玩家附属体</t>
+        </is>
+      </c>
+      <c r="J209" t="n">
+        <v>2</v>
+      </c>
+      <c r="K209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Hostile</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="J210" t="n">
+        <v>3</v>
+      </c>
+      <c r="K210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="J211" t="n">
+        <v>4</v>
+      </c>
+      <c r="K211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Pickup</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>拾取物</t>
+        </is>
+      </c>
+      <c r="J212" t="n">
+        <v>5</v>
+      </c>
+      <c r="K212" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>